<commit_message>
arima feito e no excel, machine learning next
</commit_message>
<xml_diff>
--- a/data/Bitcoin_2010_2025.xlsx
+++ b/data/Bitcoin_2010_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tiago\Desktop\ANO 3\ANO 3 SEM 2\PIC\Financial-Markets-Prediction\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A6614A-3433-478E-A577-53CBD867EF92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D483C9C-7FA2-41ED-BFC2-472687B7D071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{05E26C56-CA90-4BCB-B268-87BF101DE485}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5650" uniqueCount="4694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5654" uniqueCount="4697">
   <si>
     <t>0.1</t>
   </si>
@@ -14102,6 +14102,15 @@
   </si>
   <si>
     <t>Close</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>88,812.1</t>
   </si>
 </sst>
 </file>
@@ -14968,7 +14977,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F00219A-FBD2-48C3-BB5C-932243FD0CA8}">
-  <dimension ref="A1:D5647"/>
+  <dimension ref="A1:D5648"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.36328125" style="2" customWidth="1"/>
@@ -94035,7 +94044,24 @@
         <v>4689</v>
       </c>
     </row>
+    <row r="5648" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5648" s="2" t="s">
+        <v>4694</v>
+      </c>
+      <c r="B5648" s="2" t="s">
+        <v>4694</v>
+      </c>
+      <c r="C5648" s="2" t="s">
+        <v>4695</v>
+      </c>
+      <c r="D5648" s="1" t="s">
+        <v>4696</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A5648:C5648" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>